<commit_message>
Add PF tie-out bridge (salary REVISED_PF -> ECR EE) to pivot summary
Month-wise bridge documenting why full-sheet salary PF (FY Rs.29,17,58,299)
differs from ECR-matched figures in PF_ESI_Reco_Summary: unmatched-row PF
(FY Rs.11,14,184) and matching residual (FY Rs.5,08,332); identity to TOTAL
ECR EE checks to 0 all 12 months. Added as PF_Tieout tab in pivot xlsx,
CSV, and the Drive Google Sheet.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Rxz8VcCB74nG7vtiLVCEGq
</commit_message>
<xml_diff>
--- a/docs/salary-monthly-summary-fy2025-26/consol/PIVOT_12M_Summary_FY2025-26.xlsx
+++ b/docs/salary-monthly-summary-fy2025-26/consol/PIVOT_12M_Summary_FY2025-26.xlsx
@@ -8,8 +8,9 @@
   </bookViews>
   <sheets>
     <sheet name="Pivot_Month" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Pivot_State_NetPayable" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="README" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="PF_Tieout" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Pivot_State_NetPayable" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="README" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1844,6 +1845,550 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="44" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>MONTH</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>SALARY SHEET REVISED_PF (all rows)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>PF on rows NOT matched to ECR</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>REVISED PF (ECR-matched)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Matching residual (EE − matched)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>ECR PF matched in salary (EE)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>BACK OFFICE (ECR)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>ECR-only (not in salary)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>TOTAL PF AS PER ECR (EE)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Check (EE+BO+only − Total)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Apr-25</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>22980428</v>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>81524</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>22898904</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>60009</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>22958913</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>286145</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>9101</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>23254159</v>
+      </c>
+      <c r="J2" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>May-25</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>22977657</v>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>54050</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>22923607</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>10992</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>22934599</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>311829</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>6131</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>23252559</v>
+      </c>
+      <c r="J3" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Jun-25</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>23319453</v>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>45595</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>23273858</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>12371</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>23286229</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>302776</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>6229</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>23595234</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Jul-25</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>23982900</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>348213</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>23634687</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>310419</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>23945106</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>316353</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>11092</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>24272551</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Aug-25</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>23833745</v>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>39881</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>23793864</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>16398</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>23810262</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>332333</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>12953</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>24155548</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Sep-25</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>24402372</v>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>55422</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>24346950</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>5974</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>24352924</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>349252</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>14962</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>24717138</v>
+      </c>
+      <c r="J7" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Oct-25</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>24286578</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>61115</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>24225463</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>5165</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>24230628</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>355302</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>34681</v>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>24620611</v>
+      </c>
+      <c r="J8" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Nov-25</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>23861498</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>65500</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>23795998</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>5947</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>23801945</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>362125</v>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>30066</v>
+      </c>
+      <c r="I9" s="3" t="n">
+        <v>24194136</v>
+      </c>
+      <c r="J9" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Dec-25</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>25136852</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>63756</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>25073096</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>4457</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>25077553</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>368032</v>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>35729</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>25481314</v>
+      </c>
+      <c r="J10" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Jan-26</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>25669090</v>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>141981</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>25527109</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>60694</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>25587803</v>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>383052</v>
+      </c>
+      <c r="H11" s="3" t="n">
+        <v>13726</v>
+      </c>
+      <c r="I11" s="3" t="n">
+        <v>25984581</v>
+      </c>
+      <c r="J11" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Feb-26</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>25462898</v>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>61523</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>25401375</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>10075</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>25411450</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>364033</v>
+      </c>
+      <c r="H12" s="3" t="n">
+        <v>82343</v>
+      </c>
+      <c r="I12" s="3" t="n">
+        <v>25857826</v>
+      </c>
+      <c r="J12" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Mar-26</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>25844828</v>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>95624</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>25749204</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>5831</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>25755035</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>397142</v>
+      </c>
+      <c r="H13" s="3" t="n">
+        <v>32622</v>
+      </c>
+      <c r="I13" s="3" t="n">
+        <v>26184799</v>
+      </c>
+      <c r="J13" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>TOTAL FY 2025-26</t>
+        </is>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>291758299</v>
+      </c>
+      <c r="C14" s="6" t="n">
+        <v>1114184</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>290644115</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>508332</v>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>291152447</v>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>4128374</v>
+      </c>
+      <c r="H14" s="6" t="n">
+        <v>289635</v>
+      </c>
+      <c r="I14" s="6" t="n">
+        <v>295570456</v>
+      </c>
+      <c r="J14" s="6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Bridge: SALARY SHEET REVISED_PF − unmatched rows = matched PF; + residual = ECR EE (matched); + BACK OFFICE + ECR-only = TOTAL ECR EE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Salary-side figures from the 12-month consol (verified against source files); ECR-side from PF_ESI_Reco_Summary_FY2025-26110726.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Both views are correct: 22,980,428 (Apr) = PF deducted in the salary sheet; 22,958,913 (Apr) = ECR EE for matched employees.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:N27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3136,7 +3681,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3155,9 +3700,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -3186,9 +3729,7 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr"/>
-    </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
@@ -3210,9 +3751,7 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr"/>
-    </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -3227,9 +3766,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr"/>
-    </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
PF tie-out: correct column-C interpretation per skill (12% basic/MW-floor lift, not unmatched PF)
Row-level verification: REVISED_PF = ECR_PF anchor on all 235,082 rows; employee-
level reco shows zero amount-mismatches and only 3 salary-only PF rows (Jun-25,
Rs.4,196). The Rs.11.14L bridge item is the deliberate 12%-basic/MW-floor lift
(03-Jul) over the 02-Jul reco snapshot - per skill, ECR <= Revised, net unchanged.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Rxz8VcCB74nG7vtiLVCEGq
</commit_message>
<xml_diff>
--- a/docs/salary-monthly-summary-fy2025-26/consol/PIVOT_12M_Summary_FY2025-26.xlsx
+++ b/docs/salary-monthly-summary-fy2025-26/consol/PIVOT_12M_Summary_FY2025-26.xlsx
@@ -1845,7 +1845,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J18"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -1873,7 +1873,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>PF on rows NOT matched to ECR</t>
+          <t>12%-basic / MW-floor lift vs ECR-matched basis (skill: ECR ≤ Revised)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -2355,26 +2355,37 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr"/>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>SKILL COMPLIANCE (verified row-level on all 235,082 consol rows):</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Bridge: SALARY SHEET REVISED_PF − unmatched rows = matched PF; + residual = ECR EE (matched); + BACK OFFICE + ECR-only = TOTAL ECR EE.</t>
+          <t>1. REVISED_PF = ECR_PF anchor on EVERY row; zero rows carry PF without an ECR anchor.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Salary-side figures from the 12-month consol (verified against source files); ECR-side from PF_ESI_Reco_Summary_FY2025-26110726.</t>
+          <t>2. Employee-level reco: zero amount-mismatches where both sides have PF; only 3 employees have salary PF missing from ECR - Jun-25, Rs.4,196 (MALEK MAHMADRAFIK 1,518 / NALLOLLA KUMAR 1,236 / PURRA MANIKYAM 1,442) - flagged for review.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Both views are correct: 22,980,428 (Apr) = PF deducted in the salary sheet; 22,958,913 (Apr) = ECR EE for matched employees.</t>
+          <t>3. Column C is NOT unmatched PF: it is the deliberate 12%-basic / minimum-wage-floor lift applied 03-Jul (after the 02-Jul reco snapshot). Per the skill: ECR &lt;= Revised, excess absorbed in Other Deduction, NET unchanged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>4. Both bases correct: 22,980,428 (Apr) = final sheets after 12% fix; 22,958,913 (Apr) = ECR EE matched basis.</t>
         </is>
       </c>
     </row>
@@ -3700,7 +3711,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -3729,7 +3739,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
@@ -3751,7 +3760,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
@@ -3766,7 +3774,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Headline PF on ECR matched-EE basis in 12M pivot + dashboard
Pivot_Month column I now shows PF as per ECR (matched EE) — Apr-25
22,958,913 ... FY 291,152,447 — with the salary-sheet column sum kept
in column J as reference. Dashboard PF trend/KPI/table switched to the
same ECR basis. Presentation only: no salary-sheet data or net payable
figures were touched (net payable unchanged, Δ = 0 all months).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Rxz8VcCB74nG7vtiLVCEGq
</commit_message>
<xml_diff>
--- a/docs/salary-monthly-summary-fy2025-26/consol/PIVOT_12M_Summary_FY2025-26.xlsx
+++ b/docs/salary-monthly-summary-fy2025-26/consol/PIVOT_12M_Summary_FY2025-26.xlsx
@@ -88,7 +88,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -98,6 +98,7 @@
     <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -549,12 +550,12 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>ECR_PF</t>
+          <t>PF (AS PER ECR, MATCHED EE) ★</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>REVISED_PF</t>
+          <t>PF AS PER SALARY SHEET (col sum, ref)</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
@@ -725,8 +726,8 @@
       <c r="H2" s="3" t="n">
         <v>307258776.67</v>
       </c>
-      <c r="I2" s="3" t="n">
-        <v>22980428</v>
+      <c r="I2" s="7" t="n">
+        <v>22958913</v>
       </c>
       <c r="J2" s="3" t="n">
         <v>22980428</v>
@@ -843,8 +844,8 @@
       <c r="H3" s="3" t="n">
         <v>294937932.35</v>
       </c>
-      <c r="I3" s="3" t="n">
-        <v>22977657</v>
+      <c r="I3" s="7" t="n">
+        <v>22934599</v>
       </c>
       <c r="J3" s="3" t="n">
         <v>22977657</v>
@@ -959,8 +960,8 @@
       <c r="H4" s="3" t="n">
         <v>311862253.69</v>
       </c>
-      <c r="I4" s="3" t="n">
-        <v>23319453</v>
+      <c r="I4" s="7" t="n">
+        <v>23286229</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>23319453</v>
@@ -1071,8 +1072,8 @@
       <c r="H5" s="3" t="n">
         <v>300370600.33</v>
       </c>
-      <c r="I5" s="3" t="n">
-        <v>23982900</v>
+      <c r="I5" s="7" t="n">
+        <v>23945106</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>23982900</v>
@@ -1145,8 +1146,8 @@
       <c r="H6" s="3" t="n">
         <v>302404123.67</v>
       </c>
-      <c r="I6" s="3" t="n">
-        <v>23833745</v>
+      <c r="I6" s="7" t="n">
+        <v>23810262</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>23833745</v>
@@ -1221,8 +1222,8 @@
       <c r="H7" s="3" t="n">
         <v>302377397.67</v>
       </c>
-      <c r="I7" s="3" t="n">
-        <v>24402372</v>
+      <c r="I7" s="7" t="n">
+        <v>24352924</v>
       </c>
       <c r="J7" s="3" t="n">
         <v>24402372</v>
@@ -1297,8 +1298,8 @@
       <c r="H8" s="3" t="n">
         <v>313230127</v>
       </c>
-      <c r="I8" s="3" t="n">
-        <v>24286578</v>
+      <c r="I8" s="7" t="n">
+        <v>24230628</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>24286578</v>
@@ -1373,8 +1374,8 @@
       <c r="H9" s="3" t="n">
         <v>306692287.67</v>
       </c>
-      <c r="I9" s="3" t="n">
-        <v>23861498</v>
+      <c r="I9" s="7" t="n">
+        <v>23801945</v>
       </c>
       <c r="J9" s="3" t="n">
         <v>23861498</v>
@@ -1447,8 +1448,8 @@
       <c r="H10" s="3" t="n">
         <v>322259850.33</v>
       </c>
-      <c r="I10" s="3" t="n">
-        <v>25136852</v>
+      <c r="I10" s="7" t="n">
+        <v>25077553</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>25136852</v>
@@ -1521,8 +1522,8 @@
       <c r="H11" s="3" t="n">
         <v>330412276.33</v>
       </c>
-      <c r="I11" s="3" t="n">
-        <v>25669090</v>
+      <c r="I11" s="7" t="n">
+        <v>25587803</v>
       </c>
       <c r="J11" s="3" t="n">
         <v>25669090</v>
@@ -1595,8 +1596,8 @@
       <c r="H12" s="3" t="n">
         <v>334720608</v>
       </c>
-      <c r="I12" s="3" t="n">
-        <v>25462898</v>
+      <c r="I12" s="7" t="n">
+        <v>25411450</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>25462898</v>
@@ -1669,8 +1670,8 @@
       <c r="H13" s="3" t="n">
         <v>340340459</v>
       </c>
-      <c r="I13" s="3" t="n">
-        <v>25844828</v>
+      <c r="I13" s="7" t="n">
+        <v>25755035</v>
       </c>
       <c r="J13" s="3" t="n">
         <v>25844828</v>
@@ -1743,8 +1744,8 @@
       <c r="H14" s="6" t="n">
         <v>3766866692.71</v>
       </c>
-      <c r="I14" s="6" t="n">
-        <v>291758299</v>
+      <c r="I14" s="7" t="n">
+        <v>291152447</v>
       </c>
       <c r="J14" s="6" t="n">
         <v>291758299</v>

</xml_diff>

<commit_message>
PF tie-out: match all 12 months to Anuj EPF challan register
Anuj's PF SUMM ACCOUNTS current-month challan EE (DELHI + STEAG
BHATINDA + DMART MUMBAI + CCU HISAR + DELHI DUTY FREE, excluding
arrear/penalty rows) equals TOTAL PF AS PER ECR (EE) to the rupee in
every month, Apr-25 through Mar-26 (check = 0). Added four columns to
PF_Tieout (CSV, xlsx and the Google Sheet tab): Anuj current-month EE,
check vs ECR EE, arrear/penalty EE, and Anuj month total as deposited.
Verification only - no salary-sheet data or net payable touched.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Rxz8VcCB74nG7vtiLVCEGq
</commit_message>
<xml_diff>
--- a/docs/salary-monthly-summary-fy2025-26/consol/PIVOT_12M_Summary_FY2025-26.xlsx
+++ b/docs/salary-monthly-summary-fy2025-26/consol/PIVOT_12M_Summary_FY2025-26.xlsx
@@ -22,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[&gt;=10000000]##\,##\,##\,##0;[&gt;=100000]##\,##\,##0;#,##0"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -38,8 +38,12 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -59,6 +63,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000D5932"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9F2DE"/>
       </patternFill>
     </fill>
   </fills>
@@ -88,7 +102,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -99,6 +113,13 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1846,7 +1867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J19"/>
+  <dimension ref="A1:N20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -1859,6 +1880,10 @@
     <col width="17" customWidth="1" min="8" max="8"/>
     <col width="17" customWidth="1" min="9" max="9"/>
     <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="18" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="44" customHeight="1">
@@ -1912,6 +1937,26 @@
           <t>Check (EE+BO+only − Total)</t>
         </is>
       </c>
+      <c r="K1" s="8" t="inlineStr">
+        <is>
+          <t>ANUJ PF REGISTER: CURRENT-MONTH CHALLAN EE</t>
+        </is>
+      </c>
+      <c r="L1" s="8" t="inlineStr">
+        <is>
+          <t>Check (ECR EE − ANUJ current)</t>
+        </is>
+      </c>
+      <c r="M1" s="8" t="inlineStr">
+        <is>
+          <t>ANUJ PF REGISTER: ARREAR / PENALTY EE</t>
+        </is>
+      </c>
+      <c r="N1" s="8" t="inlineStr">
+        <is>
+          <t>ANUJ MONTH TOTAL EE (as deposited)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1946,6 +1991,18 @@
       <c r="J2" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="K2" s="9" t="n">
+        <v>23254159</v>
+      </c>
+      <c r="L2" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" s="9" t="n">
+        <v>29082</v>
+      </c>
+      <c r="N2" s="9" t="n">
+        <v>23283241</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1980,6 +2037,18 @@
       <c r="J3" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="K3" s="9" t="n">
+        <v>23252559</v>
+      </c>
+      <c r="L3" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" s="9" t="n">
+        <v>126193</v>
+      </c>
+      <c r="N3" s="9" t="n">
+        <v>23378752</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -2014,6 +2083,18 @@
       <c r="J4" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="K4" s="9" t="n">
+        <v>23595234</v>
+      </c>
+      <c r="L4" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="9" t="n">
+        <v>106948</v>
+      </c>
+      <c r="N4" s="9" t="n">
+        <v>23702182</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -2048,6 +2129,18 @@
       <c r="J5" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="K5" s="9" t="n">
+        <v>24272551</v>
+      </c>
+      <c r="L5" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" s="9" t="n">
+        <v>208348</v>
+      </c>
+      <c r="N5" s="9" t="n">
+        <v>24480899</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -2082,6 +2175,18 @@
       <c r="J6" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="K6" s="9" t="n">
+        <v>24155548</v>
+      </c>
+      <c r="L6" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="9" t="n">
+        <v>145942</v>
+      </c>
+      <c r="N6" s="9" t="n">
+        <v>24301490</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -2116,6 +2221,18 @@
       <c r="J7" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="K7" s="9" t="n">
+        <v>24717138</v>
+      </c>
+      <c r="L7" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" s="9" t="n">
+        <v>75701</v>
+      </c>
+      <c r="N7" s="9" t="n">
+        <v>24792839</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -2150,6 +2267,18 @@
       <c r="J8" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="K8" s="9" t="n">
+        <v>24620611</v>
+      </c>
+      <c r="L8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="9" t="n">
+        <v>107144</v>
+      </c>
+      <c r="N8" s="9" t="n">
+        <v>24727755</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -2184,6 +2313,18 @@
       <c r="J9" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="K9" s="9" t="n">
+        <v>24194136</v>
+      </c>
+      <c r="L9" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" s="9" t="n">
+        <v>94611</v>
+      </c>
+      <c r="N9" s="9" t="n">
+        <v>24288747</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -2218,6 +2359,18 @@
       <c r="J10" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="K10" s="9" t="n">
+        <v>25481314</v>
+      </c>
+      <c r="L10" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="9" t="n">
+        <v>130207</v>
+      </c>
+      <c r="N10" s="9" t="n">
+        <v>25611521</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -2252,6 +2405,18 @@
       <c r="J11" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="K11" s="9" t="n">
+        <v>25984581</v>
+      </c>
+      <c r="L11" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" s="9" t="n">
+        <v>84518</v>
+      </c>
+      <c r="N11" s="9" t="n">
+        <v>26069099</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2286,6 +2451,18 @@
       <c r="J12" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="K12" s="9" t="n">
+        <v>25857826</v>
+      </c>
+      <c r="L12" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="9" t="n">
+        <v>39182</v>
+      </c>
+      <c r="N12" s="9" t="n">
+        <v>25897008</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -2320,6 +2497,18 @@
       <c r="J13" s="3" t="n">
         <v>0</v>
       </c>
+      <c r="K13" s="9" t="n">
+        <v>26184799</v>
+      </c>
+      <c r="L13" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="9" t="n">
+        <v>59350</v>
+      </c>
+      <c r="N13" s="9" t="n">
+        <v>26244149</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -2354,6 +2543,18 @@
       <c r="J14" s="6" t="n">
         <v>0</v>
       </c>
+      <c r="K14" s="11" t="n">
+        <v>295570456</v>
+      </c>
+      <c r="L14" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="11" t="n">
+        <v>1207226</v>
+      </c>
+      <c r="N14" s="11" t="n">
+        <v>296777682</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2387,6 +2588,13 @@
       <c r="A19" t="inlineStr">
         <is>
           <t>4. Both bases correct: 22,980,428 (Apr) = final sheets after 12% fix; 22,958,913 (Apr) = ECR EE matched basis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>5. ANUJ PF REGISTER MATCH: current-month challan EE (all establishments, excl. arrears/penalties) = TOTAL PF AS PER ECR (EE) to the rupee in ALL 12 months (check = 0). Anuj month total = ECR EE + that month's arrear/penalty challans.</t>
         </is>
       </c>
     </row>

</xml_diff>